<commit_message>
Circle Mall feasibility: two rent scenarios over 3 years with Al Khail Avenue sales assumption
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0162jesZSmnoREDG13Pdh43J
</commit_message>
<xml_diff>
--- a/circle_mall_feasibility/Circle_Mall_Inputs.xlsx
+++ b/circle_mall_feasibility/Circle_Mall_Inputs.xlsx
@@ -23,8 +23,10 @@
     <sheet name="10 Online channels" sheetId="14" state="visible" r:id="rId14"/>
     <sheet name="11 External growth drivers" sheetId="15" state="visible" r:id="rId15"/>
     <sheet name="12 Model backtest (derived)" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="13 Monthly forecast (derived)" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="14 Lease-year P&amp;L (derived)" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="14a Lease-year P&amp;L S1 (derived)" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="14b Lease-year P&amp;L S2 (derived)" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="13 Monthly forecast (derived)" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="13b Lease-year sales (derived)" sheetId="20" state="visible" r:id="rId20"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -446,10 +448,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="31" customWidth="1" min="1" max="1"/>
+    <col width="33" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -648,7 +650,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>13 Monthly forecast (derived)</t>
+          <t>14a Lease-year P&amp;L S1 (derived)</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -660,10 +662,34 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>14 Lease-year P&amp;L (derived)</t>
+          <t>14b Lease-year P&amp;L S2 (derived)</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
+        <is>
+          <t>Derived output</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>13 Monthly forecast (derived)</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Derived output</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>13b Lease-year sales (derived)</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
         <is>
           <t>Derived output</t>
         </is>
@@ -4833,7 +4859,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Used for years 2-3 (50% blend) and years 4-5 (100%)</t>
+          <t>Reference only: not used for years 2-3, which follow the Al Khail Avenue assumption</t>
         </is>
       </c>
     </row>
@@ -5146,623 +5172,383 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B61"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="29" customWidth="1" min="3" max="3"/>
+    <col width="29" customWidth="1" min="4" max="4"/>
+    <col width="29" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Month</t>
+          <t>Line</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Forecast net sales (AED)</t>
+          <t>8 Aug 25 - 7 Aug 26 (actual, old rent)</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Year 1: 8 Aug 26 - 7 Aug 27</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Year 2: 8 Aug 27 - 7 Aug 28</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Year 3: 8 Aug 28 - 7 Aug 29</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09</t>
+          <t>Net sales</t>
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>274570.1839274962</v>
+        <v>3935572.373279454</v>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>4156573.008530711</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>4156573.008530712</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>3740915.70767764</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10</t>
+          <t>Gross margin</t>
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>326258.8097443273</v>
+        <v>2862417.050630145</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>3076214.803262552</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>3075864.026130599</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>2768277.623517538</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-11</t>
+          <t>Net Income (Income)</t>
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>386964.9318842131</v>
+        <v>2505988.343900825</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>2661443.606628563</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>2660206.728009454</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>2394186.055208508</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-12</t>
+          <t>Employee expense</t>
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>469124.2674214104</v>
+        <v>327768.4131182797</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>374925.9397849462</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>386778.5996774194</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>394514.1704301075</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2027-01</t>
+          <t>Rent (gross)</t>
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>359807.1124674876</v>
+        <v>560456.4906234774</v>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>885108.0000000001</v>
+      </c>
+      <c r="D6" t="n">
+        <v>1043420</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1093792</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2027-02</t>
+          <t>Advertising &amp; marketing</t>
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>326782.6600818752</v>
+        <v>72823.46105376343</v>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>85084.11518279569</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>92479.92430107528</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>94329.52290322582</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2027-03</t>
+          <t>Other opex</t>
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>378026.4853467933</v>
+        <v>267881.0646236559</v>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>274873.9544086021</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>284201.8482795698</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>289885.8878494623</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2027-04</t>
+          <t>Shared common</t>
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>334006.1355105379</v>
+        <v>201635.9452688172</v>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>193811.950967742</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>206114.5976344086</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>210236.890860215</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2027-05</t>
+          <t>Shared others</t>
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>399307.5354269648</v>
+        <v>96172.26969892473</v>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>85325.97470967742</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>94161.17376344085</v>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>96044.39978494625</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2027-06</t>
+          <t>Total expense</t>
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>328429.3009519565</v>
+        <v>1526737.644386918</v>
+      </c>
+      <c r="C11" s="3" t="n">
+        <v>1899129.935053763</v>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>2107156.143655914</v>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>2178802.871827957</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2027-07</t>
+          <t>Store / cash profit</t>
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>302713.1068048548</v>
+        <v>979250.6995139071</v>
+      </c>
+      <c r="C12" s="3" t="n">
+        <v>762313.6715747993</v>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>553050.5843535406</v>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>215383.1833805507</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2027-08</t>
+          <t>Depreciation</t>
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>286526.6066404763</v>
+        <v>118383.8132258064</v>
+      </c>
+      <c r="C13" s="3" t="n">
+        <v>9161.106236559141</v>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>6052.873763440861</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2027-09</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="B14" s="3" t="n">
-        <v>287578.8753687204</v>
+        <v>3813.564838709678</v>
+      </c>
+      <c r="C14" s="3" t="n">
+        <v>4002.06193548387</v>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>1940.793225806451</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2027-10</t>
+          <t>Net profit (pre-tax)</t>
         </is>
       </c>
       <c r="B15" s="3" t="n">
-        <v>339879.8663378757</v>
+        <v>857053.321449391</v>
+      </c>
+      <c r="C15" s="3" t="n">
+        <v>749150.5034027564</v>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>545056.9173642932</v>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>215383.1833805507</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2027-11</t>
+          <t>Rent / sq ft</t>
         </is>
       </c>
       <c r="B16" s="3" t="n">
-        <v>406741.8157482208</v>
+        <v>155.7688967825118</v>
+      </c>
+      <c r="C16" t="n">
+        <v>246</v>
+      </c>
+      <c r="D16" t="n">
+        <v>290</v>
+      </c>
+      <c r="E16" t="n">
+        <v>304</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2027-12</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="n">
-        <v>483639.8361106041</v>
+          <t>Rent-to-sales</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>0.1424078729764172</v>
+      </c>
+      <c r="C17" s="2" t="n">
+        <v>0.2129417667351098</v>
+      </c>
+      <c r="D17" s="2" t="n">
+        <v>0.2510289120048042</v>
+      </c>
+      <c r="E17" s="2" t="n">
+        <v>0.292386165706745</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2028-01</t>
-        </is>
-      </c>
-      <c r="B18" s="3" t="n">
-        <v>378619.6639303358</v>
+          <t>Rent-to-income</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="n">
+        <v>0.2236468864619977</v>
+      </c>
+      <c r="C18" s="2" t="n">
+        <v>0.3325668812953841</v>
+      </c>
+      <c r="D18" s="2" t="n">
+        <v>0.3922326746315528</v>
+      </c>
+      <c r="E18" s="2" t="n">
+        <v>0.4568533834788969</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2028-02</t>
+          <t>PAT (9% tax)</t>
         </is>
       </c>
       <c r="B19" s="3" t="n">
-        <v>343309.0515304079</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>2028-03</t>
-        </is>
-      </c>
-      <c r="B20" s="3" t="n">
-        <v>396559.5811438643</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>2028-04</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="n">
-        <v>349403.7197606287</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>2028-05</t>
-        </is>
-      </c>
-      <c r="B22" s="3" t="n">
-        <v>419253.1058949999</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>2028-06</t>
-        </is>
-      </c>
-      <c r="B23" s="3" t="n">
-        <v>340092.2094356074</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>2028-07</t>
-        </is>
-      </c>
-      <c r="B24" s="3" t="n">
-        <v>313095.7666461183</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>2028-08</t>
-        </is>
-      </c>
-      <c r="B25" s="3" t="n">
-        <v>298461.5862048197</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>2028-09</t>
-        </is>
-      </c>
-      <c r="B26" s="3" t="n">
-        <v>301267.5039573296</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>2028-10</t>
-        </is>
-      </c>
-      <c r="B27" s="3" t="n">
-        <v>353247.9938744739</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>2028-11</t>
-        </is>
-      </c>
-      <c r="B28" s="3" t="n">
-        <v>427967.030443542</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>2028-12</t>
-        </is>
-      </c>
-      <c r="B29" s="3" t="n">
-        <v>502707.9072793234</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>2029-01</t>
-        </is>
-      </c>
-      <c r="B30" s="3" t="n">
-        <v>398978.8561465328</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>2029-02</t>
-        </is>
-      </c>
-      <c r="B31" s="3" t="n">
-        <v>360999.5490335862</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>2029-03</t>
-        </is>
-      </c>
-      <c r="B32" s="3" t="n">
-        <v>416846.6014753393</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>2029-04</t>
-        </is>
-      </c>
-      <c r="B33" s="3" t="n">
-        <v>365845.2015227463</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>2029-05</t>
-        </is>
-      </c>
-      <c r="B34" s="3" t="n">
-        <v>439558.4252529555</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>2029-06</t>
-        </is>
-      </c>
-      <c r="B35" s="3" t="n">
-        <v>352479.4648738315</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>2029-07</t>
-        </is>
-      </c>
-      <c r="B36" s="3" t="n">
-        <v>324280.4032239768</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>2029-08</t>
-        </is>
-      </c>
-      <c r="B37" s="3" t="n">
-        <v>310370.203494392</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>2029-09</t>
-        </is>
-      </c>
-      <c r="B38" s="3" t="n">
-        <v>313288.077365227</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>2029-10</t>
-        </is>
-      </c>
-      <c r="B39" s="3" t="n">
-        <v>367342.5888300654</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>2029-11</t>
-        </is>
-      </c>
-      <c r="B40" s="3" t="n">
-        <v>445042.9149582394</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>2029-12</t>
-        </is>
-      </c>
-      <c r="B41" s="3" t="n">
-        <v>522765.9527797684</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>2030-01</t>
-        </is>
-      </c>
-      <c r="B42" s="3" t="n">
-        <v>414898.1125067795</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>2030-02</t>
-        </is>
-      </c>
-      <c r="B43" s="3" t="n">
-        <v>375403.4310400262</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>2030-03</t>
-        </is>
-      </c>
-      <c r="B44" s="3" t="n">
-        <v>433478.7808742053</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>2030-04</t>
-        </is>
-      </c>
-      <c r="B45" s="3" t="n">
-        <v>380442.425063504</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>2030-05</t>
-        </is>
-      </c>
-      <c r="B46" s="3" t="n">
-        <v>457096.8064205485</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>2030-06</t>
-        </is>
-      </c>
-      <c r="B47" s="3" t="n">
-        <v>366543.3955222974</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>2030-07</t>
-        </is>
-      </c>
-      <c r="B48" s="3" t="n">
-        <v>337219.1913126135</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>2030-08</t>
-        </is>
-      </c>
-      <c r="B49" s="3" t="n">
-        <v>322753.9746138183</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>2030-09</t>
-        </is>
-      </c>
-      <c r="B50" s="3" t="n">
-        <v>325788.2716520996</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>2030-10</t>
-        </is>
-      </c>
-      <c r="B51" s="3" t="n">
-        <v>381999.5581243851</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>2030-11</t>
-        </is>
-      </c>
-      <c r="B52" s="3" t="n">
-        <v>462800.1272650731</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>2030-12</t>
-        </is>
-      </c>
-      <c r="B53" s="3" t="n">
-        <v>543624.3142956812</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>2031-01</t>
-        </is>
-      </c>
-      <c r="B54" s="3" t="n">
-        <v>431452.5471957999</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>2031-02</t>
-        </is>
-      </c>
-      <c r="B55" s="3" t="n">
-        <v>390382.0279385233</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>2031-03</t>
-        </is>
-      </c>
-      <c r="B56" s="3" t="n">
-        <v>450774.5842310861</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>2031-04</t>
-        </is>
-      </c>
-      <c r="B57" s="3" t="n">
-        <v>395622.0778235378</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>2031-05</t>
-        </is>
-      </c>
-      <c r="B58" s="3" t="n">
-        <v>475334.9689967284</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>2031-06</t>
-        </is>
-      </c>
-      <c r="B59" s="3" t="n">
-        <v>381168.4770036371</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>2031-07</t>
-        </is>
-      </c>
-      <c r="B60" s="3" t="n">
-        <v>350674.2370459868</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>2031-08</t>
-        </is>
-      </c>
-      <c r="B61" s="3" t="n">
-        <v>335631.8582009096</v>
+        <v>779918.5225189459</v>
+      </c>
+      <c r="C19" s="3" t="n">
+        <v>681726.9580965084</v>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>496001.7948015069</v>
+      </c>
+      <c r="E19" s="3" t="n">
+        <v>195998.6968763011</v>
       </c>
     </row>
   </sheetData>
@@ -5776,16 +5562,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="31" customWidth="1" min="3" max="3"/>
-    <col width="33" customWidth="1" min="4" max="4"/>
-    <col width="33" customWidth="1" min="5" max="5"/>
-    <col width="33" customWidth="1" min="6" max="6"/>
-    <col width="33" customWidth="1" min="7" max="7"/>
+    <col width="29" customWidth="1" min="3" max="3"/>
+    <col width="29" customWidth="1" min="4" max="4"/>
+    <col width="29" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5801,27 +5585,17 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>8 Aug 26 - 7 Aug 27 (renewal)</t>
+          <t>Year 1: 8 Aug 26 - 7 Aug 27</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>8 Aug 27 - 7 Aug 28 (projected)</t>
+          <t>Year 2: 8 Aug 27 - 7 Aug 28</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>8 Aug 28 - 7 Aug 29 (projected)</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>8 Aug 29 - 7 Aug 30 (projected)</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>8 Aug 30 - 7 Aug 31 (projected)</t>
+          <t>Year 3: 8 Aug 28 - 7 Aug 29</t>
         </is>
       </c>
     </row>
@@ -5835,19 +5609,13 @@
         <v>3935572.373279454</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>4156195.912486734</v>
+        <v>4156573.008530711</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>4347395.093933357</v>
+        <v>4156573.008530712</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>4545329.565902231</v>
-      </c>
-      <c r="F2" s="3" t="n">
-        <v>4726688.215581731</v>
-      </c>
-      <c r="G2" s="3" t="n">
-        <v>4915283.075383442</v>
+        <v>3740915.70767764</v>
       </c>
     </row>
     <row r="3">
@@ -5860,19 +5628,13 @@
         <v>2862417.050630145</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>3075935.752190026</v>
+        <v>3076214.803262552</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>3217072.369320194</v>
+        <v>3075864.026130599</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>3363543.878568488</v>
-      </c>
-      <c r="F3" s="3" t="n">
-        <v>3497749.279323371</v>
-      </c>
-      <c r="G3" s="3" t="n">
-        <v>3637309.475568374</v>
+        <v>2768277.623517538</v>
       </c>
     </row>
     <row r="4">
@@ -5885,19 +5647,13 @@
         <v>2505988.343900825</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>2661202.265160186</v>
+        <v>2661443.606628563</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>2782332.862784204</v>
+        <v>2660206.728009454</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>2909010.924965704</v>
-      </c>
-      <c r="F4" s="3" t="n">
-        <v>3025080.460871836</v>
-      </c>
-      <c r="G4" s="3" t="n">
-        <v>3145781.171260622</v>
+        <v>2394186.055208508</v>
       </c>
     </row>
     <row r="5">
@@ -5918,12 +5674,6 @@
       <c r="E5" s="3" t="n">
         <v>394514.1704301075</v>
       </c>
-      <c r="F5" s="3" t="n">
-        <v>402404.4537634409</v>
-      </c>
-      <c r="G5" s="3" t="n">
-        <v>410452.5458064518</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -5935,19 +5685,13 @@
         <v>560456.4906234774</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>885108.0000000001</v>
-      </c>
-      <c r="D6" s="3" t="n">
-        <v>929363.4</v>
-      </c>
-      <c r="E6" s="3" t="n">
-        <v>975831.5700000002</v>
-      </c>
-      <c r="F6" s="3" t="n">
-        <v>1024623.3284</v>
-      </c>
-      <c r="G6" s="3" t="n">
-        <v>1075854.5308</v>
+        <v>993048.0000000001</v>
+      </c>
+      <c r="D6" t="n">
+        <v>1043420</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1093792</v>
       </c>
     </row>
     <row r="7">
@@ -5968,12 +5712,6 @@
       <c r="E7" s="3" t="n">
         <v>94329.52290322582</v>
       </c>
-      <c r="F7" s="3" t="n">
-        <v>96216.11709677421</v>
-      </c>
-      <c r="G7" s="3" t="n">
-        <v>98140.44086021507</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -5993,12 +5731,6 @@
       <c r="E8" s="3" t="n">
         <v>289885.8878494623</v>
       </c>
-      <c r="F8" s="3" t="n">
-        <v>295683.6062365591</v>
-      </c>
-      <c r="G8" s="3" t="n">
-        <v>301597.2795698925</v>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -6018,12 +5750,6 @@
       <c r="E9" s="3" t="n">
         <v>210236.890860215</v>
       </c>
-      <c r="F9" s="3" t="n">
-        <v>214441.6275268817</v>
-      </c>
-      <c r="G9" s="3" t="n">
-        <v>218730.4558064516</v>
-      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -6043,12 +5769,6 @@
       <c r="E10" s="3" t="n">
         <v>96044.39978494625</v>
       </c>
-      <c r="F10" s="3" t="n">
-        <v>97965.28741935486</v>
-      </c>
-      <c r="G10" s="3" t="n">
-        <v>99924.59268817204</v>
-      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -6060,19 +5780,13 @@
         <v>1526737.644386918</v>
       </c>
       <c r="C11" s="3" t="n">
-        <v>1899129.935053763</v>
+        <v>2007069.935053763</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>1993099.543655914</v>
+        <v>2107156.143655914</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>2060842.441827957</v>
-      </c>
-      <c r="F11" s="3" t="n">
-        <v>2131334.420443011</v>
-      </c>
-      <c r="G11" s="3" t="n">
-        <v>2204699.845531183</v>
+        <v>2178802.871827957</v>
       </c>
     </row>
     <row r="12">
@@ -6085,19 +5799,13 @@
         <v>979250.6995139071</v>
       </c>
       <c r="C12" s="3" t="n">
-        <v>762072.3301064228</v>
+        <v>654373.6715747993</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>789233.3191282898</v>
+        <v>553050.5843535406</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>848168.4831377473</v>
-      </c>
-      <c r="F12" s="3" t="n">
-        <v>893746.0404288252</v>
-      </c>
-      <c r="G12" s="3" t="n">
-        <v>941081.325729439</v>
+        <v>215383.1833805507</v>
       </c>
     </row>
     <row r="13">
@@ -6118,12 +5826,6 @@
       <c r="E13" t="n">
         <v>0</v>
       </c>
-      <c r="F13" t="n">
-        <v>0</v>
-      </c>
-      <c r="G13" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -6143,12 +5845,6 @@
       <c r="E14" t="n">
         <v>0</v>
       </c>
-      <c r="F14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G14" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -6160,19 +5856,13 @@
         <v>857053.321449391</v>
       </c>
       <c r="C15" s="3" t="n">
-        <v>748909.1619343798</v>
+        <v>641210.5034027564</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>781239.6521390425</v>
+        <v>545056.9173642932</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>848168.4831377473</v>
-      </c>
-      <c r="F15" s="3" t="n">
-        <v>893746.0404288252</v>
-      </c>
-      <c r="G15" s="3" t="n">
-        <v>941081.325729439</v>
+        <v>215383.1833805507</v>
       </c>
     </row>
     <row r="16">
@@ -6185,19 +5875,13 @@
         <v>155.7688967825118</v>
       </c>
       <c r="C16" t="n">
-        <v>246</v>
-      </c>
-      <c r="D16" s="3" t="n">
-        <v>258.3</v>
-      </c>
-      <c r="E16" s="3" t="n">
-        <v>271.215</v>
-      </c>
-      <c r="F16" s="3" t="n">
-        <v>284.7758</v>
-      </c>
-      <c r="G16" s="3" t="n">
-        <v>299.0146</v>
+        <v>276</v>
+      </c>
+      <c r="D16" t="n">
+        <v>290</v>
+      </c>
+      <c r="E16" t="n">
+        <v>304</v>
       </c>
     </row>
     <row r="17">
@@ -6210,19 +5894,13 @@
         <v>0.1424078729764172</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>0.2129610871664668</v>
+        <v>0.2389102748735378</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>0.213774773150224</v>
+        <v>0.2510289120048042</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>0.2146888483775546</v>
-      </c>
-      <c r="F17" s="2" t="n">
-        <v>0.2167740459424181</v>
-      </c>
-      <c r="G17" s="2" t="n">
-        <v>0.2188794651905318</v>
+        <v>0.292386165706745</v>
       </c>
     </row>
     <row r="18">
@@ -6235,19 +5913,13 @@
         <v>0.2236468864619977</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>0.3325970414153103</v>
+        <v>0.3731238180387236</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>0.3340230827270651</v>
+        <v>0.3922326746315528</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>0.3354513252684002</v>
-      </c>
-      <c r="F18" s="2" t="n">
-        <v>0.3387094464603764</v>
-      </c>
-      <c r="G18" s="2" t="n">
-        <v>0.3419991640324009</v>
+        <v>0.4568533834788969</v>
       </c>
     </row>
     <row r="19">
@@ -6260,19 +5932,403 @@
         <v>779918.5225189459</v>
       </c>
       <c r="C19" s="3" t="n">
-        <v>681507.3373602857</v>
+        <v>583501.5580965084</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>710928.0834465286</v>
+        <v>496001.7948015069</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>771833.3196553501</v>
-      </c>
-      <c r="F19" s="3" t="n">
-        <v>813308.896790231</v>
-      </c>
-      <c r="G19" s="3" t="n">
-        <v>856384.0064137896</v>
+        <v>195998.6968763011</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B37"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Month</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Adopted forecast net sales (AED)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n">
+        <v>274570.1839274962</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>326258.8097443273</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-11</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>386964.9318842131</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-12</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>469124.2674214104</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2027-01</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>359807.1124674876</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2027-02</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>326782.6600818752</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2027-03</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>378026.4853467933</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2027-04</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>334006.1355105379</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2027-05</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>399307.5354269648</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2027-06</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>328429.3009519565</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2027-07</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>302713.1068048548</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2027-08</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>277149.1108686349</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2027-09</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>274932.9219547831</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2027-10</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>324934.0364310956</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2027-11</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>388855.8077900308</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2027-12</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>462372.3253146974</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2028-01</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>361970.2955595726</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2028-02</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>328212.427111559</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2028-03</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>379121.3253520717</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2028-04</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>334039.0892498373</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2028-05</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>400816.928206361</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2028-06</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>325137.041983021</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2028-07</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>299327.7370089232</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2028-08</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>254930.2039344088</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2028-09</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>247918.9315857852</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2028-10</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>290694.6951656148</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2028-11</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>352182.4542899652</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2028-12</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>413688.1861976992</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2029-01</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>328327.5177105625</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2029-02</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>297073.6017782828</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2029-03</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>343031.2354151843</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2029-04</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>301061.1841499904</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2029-05</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>361721.2401828701</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2029-06</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>290062.2575935926</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2029-07</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>266856.6972722117</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2029-08</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>257513.0872851645</v>
       </c>
     </row>
   </sheetData>
@@ -6286,12 +6342,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
     <col width="46" customWidth="1" min="2" max="2"/>
-    <col width="37" customWidth="1" min="3" max="3"/>
+    <col width="56" customWidth="1" min="3" max="3"/>
     <col width="57" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
@@ -6406,51 +6462,55 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>New rent - base</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>190</v>
+          <t>Scenario 1 rent, years 1 / 2 / 3</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>246 / 290 / 304</t>
+        </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>AED / sq ft / yr</t>
+          <t>AED / sq ft / yr gross</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>P&amp;L sheet 'P &amp; L' (Base Rent)</t>
+          <t>User instruction</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>New rent - service charge</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>41</v>
+          <t>Scenario 2 rent, years 1 / 2 / 3</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>276 / 290 / 304</t>
+        </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>AED / sq ft / yr</t>
+          <t>AED / sq ft / yr gross</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>P&amp;L sheet 'P &amp; L' (Sc/ Sq ft)</t>
+          <t>User instruction</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>New rent - marketing levy</t>
+          <t>Service charge (held flat)</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>15</v>
+        <v>41</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -6459,18 +6519,18 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>P&amp;L sheet 'P &amp; L' (MKT/Sqft)</t>
+          <t>P&amp;L sheet 'P &amp; L' (Sc/ Sq ft)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>New rent - gross</t>
+          <t>Marketing levy (held flat)</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>246</v>
+        <v>15</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -6479,19 +6539,19 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Sum of the above</t>
+          <t>P&amp;L sheet 'P &amp; L' (MKT/Sqft)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Renewal term</t>
+          <t>Renewal start</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>1 year: 8 Aug 2026 - 7 Aug 2027</t>
+          <t>8 Aug 2026</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -6503,15 +6563,15 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Projection horizon</t>
+          <t>Horizon</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>lease years (to 7 Aug 2031)</t>
+          <t>lease years (to 7 Aug 2029)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -6523,155 +6583,272 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Rent growth (projected years)</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="n">
-        <v>0.05</v>
+          <t>Sales year 1</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Model forecast</t>
+        </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>per year on gross rent</t>
+          <t>weighted ensemble of 8 methods</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>User instruction</t>
+          <t>Section 2</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Turnover rent clause</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="n">
-        <v>0.12</v>
+          <t>Sales year 2</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>0</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>higher of base rent or 12% of sales</t>
+          <t>no like-for-like growth (Al Khail Avenue mall opening)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Scenario / Circle Mall Rent sheets (TOR%)</t>
+          <t>User instruction</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Tax rate used for PAT</t>
+          <t>Sales year 3</t>
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>0.09</v>
+        <v>-0.1</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>UAE corporate tax, store level</t>
+          <t>10% decline on year 2 (Al Khail Avenue mall)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Assumption (UAE CT 9%)</t>
+          <t>User instruction</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Data cut-off</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Aug-2026</t>
-        </is>
+          <t>Turnover rent clause</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>0.12</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Sep-26 excluded (partial month)</t>
+          <t>higher of base rent or 12% of sales</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>COG file</t>
+          <t>Scenario / Circle Mall Rent sheets (TOR%)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Market rent comparables</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>230 - 240</t>
-        </is>
+          <t>Tax rate used for PAT</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>0.09</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>AED / sq ft gross</t>
+          <t>UAE corporate tax, store level</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>User-verified: Apparel Group new rentals at Circle Mall</t>
+          <t>Assumption (UAE CT 9%)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Mall annual footfall</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>7500000</v>
+          <t>Data cut-off</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Aug-2026</t>
+        </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>visitors / yr</t>
+          <t>Sep-26 excluded (partial month)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>P&amp;L sheet 'notes'</t>
+          <t>COG file</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Healthy rent-to-sales ceiling</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="n">
-        <v>0.2</v>
+          <t>Market rent comparables</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>230 - 240</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>AED / sq ft gross</t>
+        </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Report assumption (apparel benchmark)</t>
+          <t>User-verified: Apparel Group new rentals at Circle Mall</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
+          <t>Mall annual footfall</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>7500000</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>visitors / yr</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>P&amp;L sheet 'notes'</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Healthy rent-to-sales ceiling</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Report assumption (apparel benchmark)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
           <t>Healthy rent-to-income ceiling</t>
         </is>
       </c>
-      <c r="B20" s="2" t="n">
+      <c r="B22" s="2" t="n">
         <v>0.32</v>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D22" t="inlineStr">
         <is>
           <t>Report assumption</t>
         </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="21" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Lease year</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Adopted sales</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Model + market trend (reference)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>8 Aug 26 - 7 Aug 27</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n">
+        <v>4156573.008530712</v>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>4156573.008530712</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>8 Aug 27 - 7 Aug 28</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>4156573.008530712</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>4347760.83810666</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>8 Aug 28 - 7 Aug 29</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>3740915.70767764</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>4545906.722645093</v>
       </c>
     </row>
   </sheetData>
@@ -6931,10 +7108,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="33" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
@@ -7109,7 +7286,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Circle Mall · new rent</t>
+          <t>Circle Mall · Scenario 1, year 1</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -7131,6 +7308,36 @@
         <v>0.2252</v>
       </c>
       <c r="H6" t="inlineStr">
+        <is>
+          <t>Size &amp; rent: P&amp;L 'notes' (Dubai Hills 244/65/20/6.10; Dubai Mall 365/80/20/9.13; Mirdif 153.18/69.81/17.38/21.41); sales: COG file</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Circle Mall · Scenario 2, year 1</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>3598</v>
+      </c>
+      <c r="C7" t="n">
+        <v>276</v>
+      </c>
+      <c r="D7" t="n">
+        <v>993048</v>
+      </c>
+      <c r="E7" t="n">
+        <v>3929621</v>
+      </c>
+      <c r="F7" t="n">
+        <v>1092</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>0.2527</v>
+      </c>
+      <c r="H7" t="inlineStr">
         <is>
           <t>Size &amp; rent: P&amp;L 'notes' (Dubai Hills 244/65/20/6.10; Dubai Mall 365/80/20/9.13; Mirdif 153.18/69.81/17.38/21.41); sales: COG file</t>
         </is>

</xml_diff>